<commit_message>
feat: make intent journeys catalog driven
</commit_message>
<xml_diff>
--- a/artifacts/anc-test/ANCFZ_Intent_Catalog_Updated.xlsx
+++ b/artifacts/anc-test/ANCFZ_Intent_Catalog_Updated.xlsx
@@ -2,17 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf45f1a4303664dce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intents" sheetId="2" r:id="R39e65abc0d034083"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signals" sheetId="3" r:id="R7dac650c41574566"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="4" r:id="Re0331dcc6d4c446b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relations" sheetId="5" r:id="Rba62839ca7ff4d54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorkflowBindings" sheetId="6" r:id="R96ccfbd9286f4d1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DocumentRequirements" sheetId="7" r:id="R7dc9391659d84764"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRMFieldMappings" sheetId="8" r:id="R9aa9407e897c4cf0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChannelCapabilities" sheetId="9" r:id="R8046a3077ff1457d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestUtterances" sheetId="10" r:id="R8e708300e3ef4319"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CatalogManifest" sheetId="11" r:id="R42ccb141ef844722"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R71673b892a3142da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intents" sheetId="2" r:id="R40b6a4180ffe4296"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signals" sheetId="3" r:id="R97b8ad50b2414020"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="4" r:id="Rb06b6164a4ca48b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relations" sheetId="5" r:id="R55f22e35624f4c6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorkflowBindings" sheetId="6" r:id="R0599b55bf24147de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JourneyRequirements" sheetId="7" r:id="R0d842aff7bbd4c36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JourneyTransitions" sheetId="8" r:id="R5284d3c0872e48f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DocumentRequirements" sheetId="9" r:id="R4ced89563a9f4a5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRMFieldMappings" sheetId="10" r:id="R726b753864f14c38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChannelCapabilities" sheetId="11" r:id="Ra9477e7dd495455e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestUtterances" sheetId="12" r:id="R13f6328b785445a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CatalogManifest" sheetId="13" r:id="Rf6dba362f3ea49e2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -179,7 +181,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="IntentsTable" displayName="IntentsTable" ref="A1:K16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="IntentsTable" displayName="IntentsTable" ref="A1:K18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="intent_key"/>
     <x:tableColumn id="2" name="display_name"/>
@@ -198,7 +200,33 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="CatalogManifestTable" displayName="CatalogManifestTable" ref="A1:B7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="ChannelCapabilitiesTable" displayName="ChannelCapabilitiesTable" ref="A1:E6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="5">
+    <x:tableColumn id="1" name="channel"/>
+    <x:tableColumn id="2" name="text"/>
+    <x:tableColumn id="3" name="postback"/>
+    <x:tableColumn id="4" name="attachment"/>
+    <x:tableColumn id="5" name="server_authenticated"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="TestUtterancesTable" displayName="TestUtterancesTable" ref="A1:E7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="5">
+    <x:tableColumn id="1" name="test_id"/>
+    <x:tableColumn id="2" name="language"/>
+    <x:tableColumn id="3" name="label"/>
+    <x:tableColumn id="4" name="utterance"/>
+    <x:tableColumn id="5" name="expected_mode"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="CatalogManifestTable" displayName="CatalogManifestTable" ref="A1:B7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="key"/>
     <x:tableColumn id="2" name="value"/>
@@ -225,7 +253,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SlotsTable" displayName="SlotsTable" ref="A1:J7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SlotsTable" displayName="SlotsTable" ref="A1:J11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="intent_key"/>
     <x:tableColumn id="2" name="slot_key"/>
@@ -258,7 +286,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="WorkflowBindingsTable" displayName="WorkflowBindingsTable" ref="A1:F16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="WorkflowBindingsTable" displayName="WorkflowBindingsTable" ref="A1:F17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="workflow_key"/>
     <x:tableColumn id="2" name="n8n_workflow_id"/>
@@ -272,7 +300,42 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="DocumentRequirementsTable" displayName="DocumentRequirementsTable" ref="A1:E9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="JourneyRequirementsTable" displayName="JourneyRequirementsTable" ref="A1:L11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="12">
+    <x:tableColumn id="1" name="intent_key"/>
+    <x:tableColumn id="2" name="requirement_key"/>
+    <x:tableColumn id="3" name="requirement_type"/>
+    <x:tableColumn id="4" name="required"/>
+    <x:tableColumn id="5" name="collection_order"/>
+    <x:tableColumn id="6" name="prompt_key"/>
+    <x:tableColumn id="7" name="validation_rule"/>
+    <x:tableColumn id="8" name="slot_key"/>
+    <x:tableColumn id="9" name="document_type"/>
+    <x:tableColumn id="10" name="fulfillment_mode"/>
+    <x:tableColumn id="11" name="source_of_truth"/>
+    <x:tableColumn id="12" name="notes"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="JourneyTransitionsTable" displayName="JourneyTransitionsTable" ref="A1:G3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="7">
+    <x:tableColumn id="1" name="source_intent_key"/>
+    <x:tableColumn id="2" name="target_intent_key"/>
+    <x:tableColumn id="3" name="activation_mode"/>
+    <x:tableColumn id="4" name="max_depth"/>
+    <x:tableColumn id="5" name="trigger_group"/>
+    <x:tableColumn id="6" name="prompt_key"/>
+    <x:tableColumn id="7" name="notes"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="DocumentRequirementsTable" displayName="DocumentRequirementsTable" ref="A1:E9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="source_key"/>
     <x:tableColumn id="2" name="document_type"/>
@@ -284,8 +347,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="CRMFieldMappingsTable" displayName="CRMFieldMappingsTable" ref="A1:F5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="CRMFieldMappingsTable" displayName="CRMFieldMappingsTable" ref="A1:F5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="provider"/>
     <x:tableColumn id="2" name="object_name"/>
@@ -293,32 +356,6 @@
     <x:tableColumn id="4" name="remote_field"/>
     <x:tableColumn id="5" name="retention_class"/>
     <x:tableColumn id="6" name="required"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="ChannelCapabilitiesTable" displayName="ChannelCapabilitiesTable" ref="A1:E6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="5">
-    <x:tableColumn id="1" name="channel"/>
-    <x:tableColumn id="2" name="text"/>
-    <x:tableColumn id="3" name="postback"/>
-    <x:tableColumn id="4" name="attachment"/>
-    <x:tableColumn id="5" name="server_authenticated"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="TestUtterancesTable" displayName="TestUtterancesTable" ref="A1:E7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="5">
-    <x:tableColumn id="1" name="test_id"/>
-    <x:tableColumn id="2" name="language"/>
-    <x:tableColumn id="3" name="label"/>
-    <x:tableColumn id="4" name="utterance"/>
-    <x:tableColumn id="5" name="expected_mode"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -552,7 +589,7 @@
         <x:v>Intent count</x:v>
       </x:c>
       <x:c r="B4" s="5" t="str">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -577,6 +614,247 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10.5" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="9.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="7.130000114440918" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="15" t="str">
+        <x:v>provider</x:v>
+      </x:c>
+      <x:c r="B1" s="15" t="str">
+        <x:v>object_name</x:v>
+      </x:c>
+      <x:c r="C1" s="15" t="str">
+        <x:v>source_field</x:v>
+      </x:c>
+      <x:c r="D1" s="15" t="str">
+        <x:v>remote_field</x:v>
+      </x:c>
+      <x:c r="E1" s="15" t="str">
+        <x:v>retention_class</x:v>
+      </x:c>
+      <x:c r="F1" s="15" t="str">
+        <x:v>required</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="16" t="str">
+        <x:v>salesforce</x:v>
+      </x:c>
+      <x:c r="B2" s="16" t="str">
+        <x:v>Lead</x:v>
+      </x:c>
+      <x:c r="C2" s="16" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="D2" s="16" t="str">
+        <x:v>Name</x:v>
+      </x:c>
+      <x:c r="E2" s="16" t="str">
+        <x:v>pii</x:v>
+      </x:c>
+      <x:c r="F2" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="16" t="str">
+        <x:v>salesforce</x:v>
+      </x:c>
+      <x:c r="B3" s="16" t="str">
+        <x:v>Lead</x:v>
+      </x:c>
+      <x:c r="C3" s="16" t="str">
+        <x:v>email</x:v>
+      </x:c>
+      <x:c r="D3" s="16" t="str">
+        <x:v>Email</x:v>
+      </x:c>
+      <x:c r="E3" s="16" t="str">
+        <x:v>pii</x:v>
+      </x:c>
+      <x:c r="F3" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>salesforce</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>Lead</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>phone</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="str">
+        <x:v>Phone</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
+        <x:v>pii</x:v>
+      </x:c>
+      <x:c r="F4" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="16" t="str">
+        <x:v>salesforce</x:v>
+      </x:c>
+      <x:c r="B5" s="16" t="str">
+        <x:v>Lead</x:v>
+      </x:c>
+      <x:c r="C5" s="16" t="str">
+        <x:v>summary</x:v>
+      </x:c>
+      <x:c r="D5" s="16" t="str">
+        <x:v>Description</x:v>
+      </x:c>
+      <x:c r="E5" s="16" t="str">
+        <x:v>business_context</x:v>
+      </x:c>
+      <x:c r="F5" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10636cf550f6486f"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="7.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="3.5" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="7.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="9.25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16.8799991607666" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="15" t="str">
+        <x:v>channel</x:v>
+      </x:c>
+      <x:c r="B1" s="15" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="C1" s="15" t="str">
+        <x:v>postback</x:v>
+      </x:c>
+      <x:c r="D1" s="15" t="str">
+        <x:v>attachment</x:v>
+      </x:c>
+      <x:c r="E1" s="15" t="str">
+        <x:v>server_authenticated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="16" t="str">
+        <x:v>web</x:v>
+      </x:c>
+      <x:c r="B2" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C2" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D2" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E2" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="16" t="str">
+        <x:v>whatsapp</x:v>
+      </x:c>
+      <x:c r="B3" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C3" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D3" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E3" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>email</x:v>
+      </x:c>
+      <x:c r="B4" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C4" s="17" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D4" s="17" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E4" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="16" t="str">
+        <x:v>sms</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="16" t="str">
+        <x:v>voice</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9a8a1dead6542ce"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -709,12 +987,12 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b33451460cf4078"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83988e6cce6a409e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -781,7 +1059,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6cb484520cc4ad3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e4dd82e0e724faf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -791,9 +1069,9 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="16.3799991607666" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22.8799991607666" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24.6299991607666" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="91.75" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="7.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="9.380000114440918" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="22.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12.880000114440918" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="17.1299991607666" hidden="0" customWidth="1"/>
@@ -1363,10 +1641,80 @@
         <x:v>Compatibility mapping for existing CRM slots; inactive until workflow and consent review.</x:v>
       </x:c>
     </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="16" t="str">
+        <x:v>document.intake</x:v>
+      </x:c>
+      <x:c r="B17" s="16" t="str">
+        <x:v>Submit supporting documents</x:v>
+      </x:c>
+      <x:c r="C17" s="16" t="str">
+        <x:v>Collect a catalog-authorized document after an active request asks for it.</x:v>
+      </x:c>
+      <x:c r="D17" s="16" t="str">
+        <x:v>support</x:v>
+      </x:c>
+      <x:c r="E17" s="16" t="str">
+        <x:v>document.intake</x:v>
+      </x:c>
+      <x:c r="F17" s="16" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="G17" s="16" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="H17" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I17" s="17" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J17" s="16" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="K17" s="16" t="str">
+        <x:v>Compatibility mapping for the document workflow; inactive until policy and OCR review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="16" t="str">
+        <x:v>knowledge.enquiry</x:v>
+      </x:c>
+      <x:c r="B18" s="16" t="str">
+        <x:v>Ask about approved information</x:v>
+      </x:c>
+      <x:c r="C18" s="16" t="str">
+        <x:v>Answer source-grounded questions without creating a sales action.</x:v>
+      </x:c>
+      <x:c r="D18" s="16" t="str">
+        <x:v>information</x:v>
+      </x:c>
+      <x:c r="E18" s="16" t="str">
+        <x:v>human.review</x:v>
+      </x:c>
+      <x:c r="F18" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G18" s="16" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="H18" s="17" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I18" s="17" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J18" s="16" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="K18" s="16" t="str">
+        <x:v>Knowledge-only route; inactive until a tenant-approved review binding is configured.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08f1df8d57ff4bdc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5acccd6a7755457f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7073,7 +7421,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94655c76bc2f4f93"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e74fbed23f74abf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7083,13 +7431,13 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="16.3799991607666" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="10.880000114440918" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="7.130000114440918" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="14.25" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="17.5" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="12.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17.8799991607666" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="16.8799991607666" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
   </x:cols>
@@ -7167,11 +7515,9 @@
         <x:v>email</x:v>
       </x:c>
       <x:c r="D3" s="17" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E3" s="16" t="str">
-        <x:v>contact</x:v>
-      </x:c>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E3" s="16" t="str"/>
       <x:c r="F3" s="16" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -7199,11 +7545,9 @@
         <x:v>phone</x:v>
       </x:c>
       <x:c r="D4" s="17" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E4" s="16" t="str">
-        <x:v>contact</x:v>
-      </x:c>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str"/>
       <x:c r="F4" s="16" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -7310,10 +7654,130 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="16" t="str">
+        <x:v>appointment.request</x:v>
+      </x:c>
+      <x:c r="B8" s="16" t="str">
+        <x:v>contact_consent</x:v>
+      </x:c>
+      <x:c r="C8" s="16" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D8" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E8" s="16" t="str"/>
+      <x:c r="F8" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G8" s="16" t="str">
+        <x:v>lead.ask_consent</x:v>
+      </x:c>
+      <x:c r="H8" s="16" t="str">
+        <x:v>boolean:explicit_opt_in</x:v>
+      </x:c>
+      <x:c r="I8" s="16" t="str">
+        <x:v>consent</x:v>
+      </x:c>
+      <x:c r="J8" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="16" t="str">
+        <x:v>lead.capture</x:v>
+      </x:c>
+      <x:c r="B9" s="16" t="str">
+        <x:v>interest_summary</x:v>
+      </x:c>
+      <x:c r="C9" s="16" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D9" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E9" s="16" t="str"/>
+      <x:c r="F9" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G9" s="16" t="str">
+        <x:v>lead.ask_interest</x:v>
+      </x:c>
+      <x:c r="H9" s="16" t="str">
+        <x:v>text:nonempty</x:v>
+      </x:c>
+      <x:c r="I9" s="16" t="str">
+        <x:v>business</x:v>
+      </x:c>
+      <x:c r="J9" s="16" t="n">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="16" t="str">
+        <x:v>lead.capture</x:v>
+      </x:c>
+      <x:c r="B10" s="16" t="str">
+        <x:v>contact_consent</x:v>
+      </x:c>
+      <x:c r="C10" s="16" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D10" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E10" s="16" t="str"/>
+      <x:c r="F10" s="16" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G10" s="16" t="str">
+        <x:v>lead.ask_consent</x:v>
+      </x:c>
+      <x:c r="H10" s="16" t="str">
+        <x:v>boolean:explicit_opt_in</x:v>
+      </x:c>
+      <x:c r="I10" s="16" t="str">
+        <x:v>consent</x:v>
+      </x:c>
+      <x:c r="J10" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="16" t="str">
+        <x:v>document.intake</x:v>
+      </x:c>
+      <x:c r="B11" s="16" t="str">
+        <x:v>document_consent</x:v>
+      </x:c>
+      <x:c r="C11" s="16" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D11" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E11" s="16" t="str"/>
+      <x:c r="F11" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G11" s="16" t="str">
+        <x:v>document.ask_consent</x:v>
+      </x:c>
+      <x:c r="H11" s="16" t="str">
+        <x:v>boolean:explicit_opt_in</x:v>
+      </x:c>
+      <x:c r="I11" s="16" t="str">
+        <x:v>consent</x:v>
+      </x:c>
+      <x:c r="J11" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd6825c28b4f41c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02eb32a851ab4d67"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7403,7 +7867,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cde2877441d4adb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra123752d7bc14614"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7482,16 +7946,16 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="16" t="str">
-        <x:v>anc.ancfz.int.01.request</x:v>
+        <x:v>human.review</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str">
-        <x:v>not-imported</x:v>
+        <x:v>future-managed-id</x:v>
       </x:c>
       <x:c r="C4" s="16" t="str">
-        <x:v>intent-ancfz-int-01</x:v>
+        <x:v>human-review</x:v>
       </x:c>
       <x:c r="D4" s="16" t="str">
-        <x:v>omnichannel-intent-v1</x:v>
+        <x:v>human-review-v1</x:v>
       </x:c>
       <x:c r="E4" s="16" t="str">
         <x:v>human_review</x:v>
@@ -7502,13 +7966,13 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="16" t="str">
-        <x:v>anc.ancfz.int.02.request</x:v>
+        <x:v>anc.ancfz.int.01.request</x:v>
       </x:c>
       <x:c r="B5" s="16" t="str">
         <x:v>not-imported</x:v>
       </x:c>
       <x:c r="C5" s="16" t="str">
-        <x:v>intent-ancfz-int-02</x:v>
+        <x:v>intent-ancfz-int-01</x:v>
       </x:c>
       <x:c r="D5" s="16" t="str">
         <x:v>omnichannel-intent-v1</x:v>
@@ -7522,13 +7986,13 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="16" t="str">
-        <x:v>anc.ancfz.int.03.request</x:v>
+        <x:v>anc.ancfz.int.02.request</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str">
         <x:v>not-imported</x:v>
       </x:c>
       <x:c r="C6" s="16" t="str">
-        <x:v>intent-ancfz-int-03</x:v>
+        <x:v>intent-ancfz-int-02</x:v>
       </x:c>
       <x:c r="D6" s="16" t="str">
         <x:v>omnichannel-intent-v1</x:v>
@@ -7542,13 +8006,13 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="16" t="str">
-        <x:v>anc.ancfz.int.04.request</x:v>
+        <x:v>anc.ancfz.int.03.request</x:v>
       </x:c>
       <x:c r="B7" s="16" t="str">
         <x:v>not-imported</x:v>
       </x:c>
       <x:c r="C7" s="16" t="str">
-        <x:v>intent-ancfz-int-04</x:v>
+        <x:v>intent-ancfz-int-03</x:v>
       </x:c>
       <x:c r="D7" s="16" t="str">
         <x:v>omnichannel-intent-v1</x:v>
@@ -7562,13 +8026,13 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="16" t="str">
-        <x:v>anc.ancfz.int.05.request</x:v>
+        <x:v>anc.ancfz.int.04.request</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
         <x:v>not-imported</x:v>
       </x:c>
       <x:c r="C8" s="16" t="str">
-        <x:v>intent-ancfz-int-05</x:v>
+        <x:v>intent-ancfz-int-04</x:v>
       </x:c>
       <x:c r="D8" s="16" t="str">
         <x:v>omnichannel-intent-v1</x:v>
@@ -7582,13 +8046,13 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="16" t="str">
-        <x:v>anc.ancfz.int.06.request</x:v>
+        <x:v>anc.ancfz.int.05.request</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
         <x:v>not-imported</x:v>
       </x:c>
       <x:c r="C9" s="16" t="str">
-        <x:v>intent-ancfz-int-06</x:v>
+        <x:v>intent-ancfz-int-05</x:v>
       </x:c>
       <x:c r="D9" s="16" t="str">
         <x:v>omnichannel-intent-v1</x:v>
@@ -7602,13 +8066,13 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="16" t="str">
-        <x:v>anc.ancfz.int.07.request</x:v>
+        <x:v>anc.ancfz.int.06.request</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
         <x:v>not-imported</x:v>
       </x:c>
       <x:c r="C10" s="16" t="str">
-        <x:v>intent-ancfz-int-07</x:v>
+        <x:v>intent-ancfz-int-06</x:v>
       </x:c>
       <x:c r="D10" s="16" t="str">
         <x:v>omnichannel-intent-v1</x:v>
@@ -7622,13 +8086,13 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="16" t="str">
-        <x:v>anc.ancfz.int.08.request</x:v>
+        <x:v>anc.ancfz.int.07.request</x:v>
       </x:c>
       <x:c r="B11" s="16" t="str">
         <x:v>not-imported</x:v>
       </x:c>
       <x:c r="C11" s="16" t="str">
-        <x:v>intent-ancfz-int-08</x:v>
+        <x:v>intent-ancfz-int-07</x:v>
       </x:c>
       <x:c r="D11" s="16" t="str">
         <x:v>omnichannel-intent-v1</x:v>
@@ -7642,13 +8106,13 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="16" t="str">
-        <x:v>anc.ancfz.int.09.request</x:v>
+        <x:v>anc.ancfz.int.08.request</x:v>
       </x:c>
       <x:c r="B12" s="16" t="str">
         <x:v>not-imported</x:v>
       </x:c>
       <x:c r="C12" s="16" t="str">
-        <x:v>intent-ancfz-int-09</x:v>
+        <x:v>intent-ancfz-int-08</x:v>
       </x:c>
       <x:c r="D12" s="16" t="str">
         <x:v>omnichannel-intent-v1</x:v>
@@ -7662,13 +8126,13 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="16" t="str">
-        <x:v>anc.ancfz.int.10.request</x:v>
+        <x:v>anc.ancfz.int.09.request</x:v>
       </x:c>
       <x:c r="B13" s="16" t="str">
         <x:v>not-imported</x:v>
       </x:c>
       <x:c r="C13" s="16" t="str">
-        <x:v>intent-ancfz-int-10</x:v>
+        <x:v>intent-ancfz-int-09</x:v>
       </x:c>
       <x:c r="D13" s="16" t="str">
         <x:v>omnichannel-intent-v1</x:v>
@@ -7682,13 +8146,13 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="16" t="str">
-        <x:v>anc.ancfz.int.11.request</x:v>
+        <x:v>anc.ancfz.int.10.request</x:v>
       </x:c>
       <x:c r="B14" s="16" t="str">
         <x:v>not-imported</x:v>
       </x:c>
       <x:c r="C14" s="16" t="str">
-        <x:v>intent-ancfz-int-11</x:v>
+        <x:v>intent-ancfz-int-10</x:v>
       </x:c>
       <x:c r="D14" s="16" t="str">
         <x:v>omnichannel-intent-v1</x:v>
@@ -7702,13 +8166,13 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="16" t="str">
-        <x:v>anc.ancfz.int.12.request</x:v>
+        <x:v>anc.ancfz.int.11.request</x:v>
       </x:c>
       <x:c r="B15" s="16" t="str">
         <x:v>not-imported</x:v>
       </x:c>
       <x:c r="C15" s="16" t="str">
-        <x:v>intent-ancfz-int-12</x:v>
+        <x:v>intent-ancfz-int-11</x:v>
       </x:c>
       <x:c r="D15" s="16" t="str">
         <x:v>omnichannel-intent-v1</x:v>
@@ -7722,13 +8186,13 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="16" t="str">
-        <x:v>anc.ancfz.int.13.request</x:v>
+        <x:v>anc.ancfz.int.12.request</x:v>
       </x:c>
       <x:c r="B16" s="16" t="str">
         <x:v>not-imported</x:v>
       </x:c>
       <x:c r="C16" s="16" t="str">
-        <x:v>intent-ancfz-int-13</x:v>
+        <x:v>intent-ancfz-int-12</x:v>
       </x:c>
       <x:c r="D16" s="16" t="str">
         <x:v>omnichannel-intent-v1</x:v>
@@ -7737,18 +8201,552 @@
         <x:v>human_review</x:v>
       </x:c>
       <x:c r="F16" s="17" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="16" t="str">
+        <x:v>anc.ancfz.int.13.request</x:v>
+      </x:c>
+      <x:c r="B17" s="16" t="str">
+        <x:v>not-imported</x:v>
+      </x:c>
+      <x:c r="C17" s="16" t="str">
+        <x:v>intent-ancfz-int-13</x:v>
+      </x:c>
+      <x:c r="D17" s="16" t="str">
+        <x:v>omnichannel-intent-v1</x:v>
+      </x:c>
+      <x:c r="E17" s="16" t="str">
+        <x:v>human_review</x:v>
+      </x:c>
+      <x:c r="F17" s="17" t="b">
         <x:v>0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3804cdadc18b4077"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bd541f5e2a94e30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22.6299991607666" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="7.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17.8799991607666" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="15.25" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="12.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="34.630001068115234" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="15" t="str">
+        <x:v>intent_key</x:v>
+      </x:c>
+      <x:c r="B1" s="15" t="str">
+        <x:v>requirement_key</x:v>
+      </x:c>
+      <x:c r="C1" s="15" t="str">
+        <x:v>requirement_type</x:v>
+      </x:c>
+      <x:c r="D1" s="15" t="str">
+        <x:v>required</x:v>
+      </x:c>
+      <x:c r="E1" s="15" t="str">
+        <x:v>collection_order</x:v>
+      </x:c>
+      <x:c r="F1" s="15" t="str">
+        <x:v>prompt_key</x:v>
+      </x:c>
+      <x:c r="G1" s="15" t="str">
+        <x:v>validation_rule</x:v>
+      </x:c>
+      <x:c r="H1" s="15" t="str">
+        <x:v>slot_key</x:v>
+      </x:c>
+      <x:c r="I1" s="15" t="str">
+        <x:v>document_type</x:v>
+      </x:c>
+      <x:c r="J1" s="15" t="str">
+        <x:v>fulfillment_mode</x:v>
+      </x:c>
+      <x:c r="K1" s="15" t="str">
+        <x:v>source_of_truth</x:v>
+      </x:c>
+      <x:c r="L1" s="15" t="str">
+        <x:v>notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="16" t="str">
+        <x:v>lead.capture</x:v>
+      </x:c>
+      <x:c r="B2" s="16" t="str">
+        <x:v>lead.interest-summary</x:v>
+      </x:c>
+      <x:c r="C2" s="16" t="str">
+        <x:v>slot</x:v>
+      </x:c>
+      <x:c r="D2" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E2" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F2" s="16" t="str">
+        <x:v>lead.ask_interest</x:v>
+      </x:c>
+      <x:c r="G2" s="16" t="str">
+        <x:v>text:nonempty</x:v>
+      </x:c>
+      <x:c r="H2" s="16" t="str">
+        <x:v>interest_summary</x:v>
+      </x:c>
+      <x:c r="I2" s="16" t="str"/>
+      <x:c r="J2" s="16" t="str">
+        <x:v>conversation_ready</x:v>
+      </x:c>
+      <x:c r="K2" s="16" t="str">
+        <x:v>tenant_catalog</x:v>
+      </x:c>
+      <x:c r="L2" s="16" t="str">
+        <x:v>Visitor-supplied request context.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="16" t="str">
+        <x:v>lead.capture</x:v>
+      </x:c>
+      <x:c r="B3" s="16" t="str">
+        <x:v>lead.name</x:v>
+      </x:c>
+      <x:c r="C3" s="16" t="str">
+        <x:v>slot</x:v>
+      </x:c>
+      <x:c r="D3" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E3" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F3" s="16" t="str">
+        <x:v>lead.ask_name</x:v>
+      </x:c>
+      <x:c r="G3" s="16" t="str">
+        <x:v>token:NAME</x:v>
+      </x:c>
+      <x:c r="H3" s="16" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="I3" s="16" t="str"/>
+      <x:c r="J3" s="16" t="str">
+        <x:v>conversation_ready</x:v>
+      </x:c>
+      <x:c r="K3" s="16" t="str">
+        <x:v>tenant_catalog</x:v>
+      </x:c>
+      <x:c r="L3" s="16" t="str">
+        <x:v>Validated visitor name.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>lead.capture</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>lead.email</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>slot</x:v>
+      </x:c>
+      <x:c r="D4" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F4" s="16" t="str">
+        <x:v>lead.ask_contact</x:v>
+      </x:c>
+      <x:c r="G4" s="16" t="str">
+        <x:v>token:EMAIL</x:v>
+      </x:c>
+      <x:c r="H4" s="16" t="str">
+        <x:v>email</x:v>
+      </x:c>
+      <x:c r="I4" s="16" t="str"/>
+      <x:c r="J4" s="16" t="str">
+        <x:v>conversation_ready</x:v>
+      </x:c>
+      <x:c r="K4" s="16" t="str">
+        <x:v>tenant_catalog</x:v>
+      </x:c>
+      <x:c r="L4" s="16" t="str">
+        <x:v>Validated visitor email.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="16" t="str">
+        <x:v>lead.capture</x:v>
+      </x:c>
+      <x:c r="B5" s="16" t="str">
+        <x:v>lead.phone</x:v>
+      </x:c>
+      <x:c r="C5" s="16" t="str">
+        <x:v>slot</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E5" s="16" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F5" s="16" t="str">
+        <x:v>lead.ask_contact</x:v>
+      </x:c>
+      <x:c r="G5" s="16" t="str">
+        <x:v>token:PHONE</x:v>
+      </x:c>
+      <x:c r="H5" s="16" t="str">
+        <x:v>phone</x:v>
+      </x:c>
+      <x:c r="I5" s="16" t="str"/>
+      <x:c r="J5" s="16" t="str">
+        <x:v>conversation_ready</x:v>
+      </x:c>
+      <x:c r="K5" s="16" t="str">
+        <x:v>tenant_catalog</x:v>
+      </x:c>
+      <x:c r="L5" s="16" t="str">
+        <x:v>Validated visitor phone.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="16" t="str">
+        <x:v>lead.capture</x:v>
+      </x:c>
+      <x:c r="B6" s="16" t="str">
+        <x:v>lead.contact-consent</x:v>
+      </x:c>
+      <x:c r="C6" s="16" t="str">
+        <x:v>consent</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E6" s="16" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F6" s="16" t="str">
+        <x:v>lead.ask_consent</x:v>
+      </x:c>
+      <x:c r="G6" s="16" t="str">
+        <x:v>boolean:explicit_opt_in</x:v>
+      </x:c>
+      <x:c r="H6" s="16" t="str">
+        <x:v>contact_consent</x:v>
+      </x:c>
+      <x:c r="I6" s="16" t="str"/>
+      <x:c r="J6" s="16" t="str">
+        <x:v>conversation_ready</x:v>
+      </x:c>
+      <x:c r="K6" s="16" t="str">
+        <x:v>tenant_catalog</x:v>
+      </x:c>
+      <x:c r="L6" s="16" t="str">
+        <x:v>Explicit purpose-bound contact consent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="16" t="str">
+        <x:v>appointment.request</x:v>
+      </x:c>
+      <x:c r="B7" s="16" t="str">
+        <x:v>appointment.name</x:v>
+      </x:c>
+      <x:c r="C7" s="16" t="str">
+        <x:v>slot</x:v>
+      </x:c>
+      <x:c r="D7" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E7" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F7" s="16" t="str">
+        <x:v>lead.ask_name</x:v>
+      </x:c>
+      <x:c r="G7" s="16" t="str">
+        <x:v>token:NAME</x:v>
+      </x:c>
+      <x:c r="H7" s="16" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="I7" s="16" t="str"/>
+      <x:c r="J7" s="16" t="str">
+        <x:v>conversation_ready</x:v>
+      </x:c>
+      <x:c r="K7" s="16" t="str">
+        <x:v>tenant_catalog</x:v>
+      </x:c>
+      <x:c r="L7" s="16" t="str">
+        <x:v>Validated visitor name.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="16" t="str">
+        <x:v>appointment.request</x:v>
+      </x:c>
+      <x:c r="B8" s="16" t="str">
+        <x:v>appointment.email</x:v>
+      </x:c>
+      <x:c r="C8" s="16" t="str">
+        <x:v>slot</x:v>
+      </x:c>
+      <x:c r="D8" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E8" s="16" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F8" s="16" t="str">
+        <x:v>lead.ask_contact</x:v>
+      </x:c>
+      <x:c r="G8" s="16" t="str">
+        <x:v>token:EMAIL</x:v>
+      </x:c>
+      <x:c r="H8" s="16" t="str">
+        <x:v>email</x:v>
+      </x:c>
+      <x:c r="I8" s="16" t="str"/>
+      <x:c r="J8" s="16" t="str">
+        <x:v>conversation_ready</x:v>
+      </x:c>
+      <x:c r="K8" s="16" t="str">
+        <x:v>tenant_catalog</x:v>
+      </x:c>
+      <x:c r="L8" s="16" t="str">
+        <x:v>Validated visitor email.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="16" t="str">
+        <x:v>appointment.request</x:v>
+      </x:c>
+      <x:c r="B9" s="16" t="str">
+        <x:v>appointment.time</x:v>
+      </x:c>
+      <x:c r="C9" s="16" t="str">
+        <x:v>slot</x:v>
+      </x:c>
+      <x:c r="D9" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E9" s="16" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F9" s="16" t="str">
+        <x:v>appointment.ask_time</x:v>
+      </x:c>
+      <x:c r="G9" s="16" t="str">
+        <x:v>datetime:future</x:v>
+      </x:c>
+      <x:c r="H9" s="16" t="str">
+        <x:v>meeting_time</x:v>
+      </x:c>
+      <x:c r="I9" s="16" t="str"/>
+      <x:c r="J9" s="16" t="str">
+        <x:v>conversation_ready</x:v>
+      </x:c>
+      <x:c r="K9" s="16" t="str">
+        <x:v>tenant_catalog</x:v>
+      </x:c>
+      <x:c r="L9" s="16" t="str">
+        <x:v>Visitor-supplied requested meeting time.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="16" t="str">
+        <x:v>appointment.request</x:v>
+      </x:c>
+      <x:c r="B10" s="16" t="str">
+        <x:v>appointment.contact-consent</x:v>
+      </x:c>
+      <x:c r="C10" s="16" t="str">
+        <x:v>consent</x:v>
+      </x:c>
+      <x:c r="D10" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E10" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F10" s="16" t="str">
+        <x:v>lead.ask_consent</x:v>
+      </x:c>
+      <x:c r="G10" s="16" t="str">
+        <x:v>boolean:explicit_opt_in</x:v>
+      </x:c>
+      <x:c r="H10" s="16" t="str">
+        <x:v>contact_consent</x:v>
+      </x:c>
+      <x:c r="I10" s="16" t="str"/>
+      <x:c r="J10" s="16" t="str">
+        <x:v>conversation_ready</x:v>
+      </x:c>
+      <x:c r="K10" s="16" t="str">
+        <x:v>tenant_catalog</x:v>
+      </x:c>
+      <x:c r="L10" s="16" t="str">
+        <x:v>Explicit purpose-bound appointment consent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="16" t="str">
+        <x:v>document.intake</x:v>
+      </x:c>
+      <x:c r="B11" s="16" t="str">
+        <x:v>document.upload-consent</x:v>
+      </x:c>
+      <x:c r="C11" s="16" t="str">
+        <x:v>consent</x:v>
+      </x:c>
+      <x:c r="D11" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E11" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F11" s="16" t="str">
+        <x:v>document.ask_consent</x:v>
+      </x:c>
+      <x:c r="G11" s="16" t="str">
+        <x:v>boolean:explicit_opt_in</x:v>
+      </x:c>
+      <x:c r="H11" s="16" t="str">
+        <x:v>document_consent</x:v>
+      </x:c>
+      <x:c r="I11" s="16" t="str"/>
+      <x:c r="J11" s="16" t="str">
+        <x:v>conversation_ready</x:v>
+      </x:c>
+      <x:c r="K11" s="16" t="str">
+        <x:v>tenant_catalog</x:v>
+      </x:c>
+      <x:c r="L11" s="16" t="str">
+        <x:v>Explicit document-processing consent.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c1195640a794ebd"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="13.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="9.25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.8799991607666" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20.75" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="52" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="15" t="str">
+        <x:v>source_intent_key</x:v>
+      </x:c>
+      <x:c r="B1" s="15" t="str">
+        <x:v>target_intent_key</x:v>
+      </x:c>
+      <x:c r="C1" s="15" t="str">
+        <x:v>activation_mode</x:v>
+      </x:c>
+      <x:c r="D1" s="15" t="str">
+        <x:v>max_depth</x:v>
+      </x:c>
+      <x:c r="E1" s="15" t="str">
+        <x:v>trigger_group</x:v>
+      </x:c>
+      <x:c r="F1" s="15" t="str">
+        <x:v>prompt_key</x:v>
+      </x:c>
+      <x:c r="G1" s="15" t="str">
+        <x:v>notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="16" t="str">
+        <x:v>lead.capture</x:v>
+      </x:c>
+      <x:c r="B2" s="16" t="str">
+        <x:v>appointment.request</x:v>
+      </x:c>
+      <x:c r="C2" s="16" t="str">
+        <x:v>offer</x:v>
+      </x:c>
+      <x:c r="D2" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E2" s="16" t="str">
+        <x:v>appointment_request</x:v>
+      </x:c>
+      <x:c r="F2" s="16" t="str">
+        <x:v>journey.offer_appointment</x:v>
+      </x:c>
+      <x:c r="G2" s="16" t="str">
+        <x:v>Offer appointment scheduling after the lead journey is fulfilled.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="16" t="str">
+        <x:v>appointment.request</x:v>
+      </x:c>
+      <x:c r="B3" s="16" t="str">
+        <x:v>document.intake</x:v>
+      </x:c>
+      <x:c r="C3" s="16" t="str">
+        <x:v>offer</x:v>
+      </x:c>
+      <x:c r="D3" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E3" s="16" t="str">
+        <x:v>supporting_documents</x:v>
+      </x:c>
+      <x:c r="F3" s="16" t="str">
+        <x:v>journey.offer_documents</x:v>
+      </x:c>
+      <x:c r="G3" s="16" t="str">
+        <x:v>Offer document intake only after the appointment journey is fulfilled.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ce005fd68114132"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -7915,248 +8913,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4d3c0e43715457d"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10.5" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="9.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="10.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="13.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="7.130000114440918" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="15" t="str">
-        <x:v>provider</x:v>
-      </x:c>
-      <x:c r="B1" s="15" t="str">
-        <x:v>object_name</x:v>
-      </x:c>
-      <x:c r="C1" s="15" t="str">
-        <x:v>source_field</x:v>
-      </x:c>
-      <x:c r="D1" s="15" t="str">
-        <x:v>remote_field</x:v>
-      </x:c>
-      <x:c r="E1" s="15" t="str">
-        <x:v>retention_class</x:v>
-      </x:c>
-      <x:c r="F1" s="15" t="str">
-        <x:v>required</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="16" t="str">
-        <x:v>salesforce</x:v>
-      </x:c>
-      <x:c r="B2" s="16" t="str">
-        <x:v>Lead</x:v>
-      </x:c>
-      <x:c r="C2" s="16" t="str">
-        <x:v>name</x:v>
-      </x:c>
-      <x:c r="D2" s="16" t="str">
-        <x:v>Name</x:v>
-      </x:c>
-      <x:c r="E2" s="16" t="str">
-        <x:v>pii</x:v>
-      </x:c>
-      <x:c r="F2" s="17" t="b">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="16" t="str">
-        <x:v>salesforce</x:v>
-      </x:c>
-      <x:c r="B3" s="16" t="str">
-        <x:v>Lead</x:v>
-      </x:c>
-      <x:c r="C3" s="16" t="str">
-        <x:v>email</x:v>
-      </x:c>
-      <x:c r="D3" s="16" t="str">
-        <x:v>Email</x:v>
-      </x:c>
-      <x:c r="E3" s="16" t="str">
-        <x:v>pii</x:v>
-      </x:c>
-      <x:c r="F3" s="17" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="16" t="str">
-        <x:v>salesforce</x:v>
-      </x:c>
-      <x:c r="B4" s="16" t="str">
-        <x:v>Lead</x:v>
-      </x:c>
-      <x:c r="C4" s="16" t="str">
-        <x:v>phone</x:v>
-      </x:c>
-      <x:c r="D4" s="16" t="str">
-        <x:v>Phone</x:v>
-      </x:c>
-      <x:c r="E4" s="16" t="str">
-        <x:v>pii</x:v>
-      </x:c>
-      <x:c r="F4" s="17" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="16" t="str">
-        <x:v>salesforce</x:v>
-      </x:c>
-      <x:c r="B5" s="16" t="str">
-        <x:v>Lead</x:v>
-      </x:c>
-      <x:c r="C5" s="16" t="str">
-        <x:v>summary</x:v>
-      </x:c>
-      <x:c r="D5" s="16" t="str">
-        <x:v>Description</x:v>
-      </x:c>
-      <x:c r="E5" s="16" t="str">
-        <x:v>business_context</x:v>
-      </x:c>
-      <x:c r="F5" s="17" t="b">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd37259a1ca9c4b9b"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="7.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="3.5" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="7.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="9.25" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16.8799991607666" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="15" t="str">
-        <x:v>channel</x:v>
-      </x:c>
-      <x:c r="B1" s="15" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="C1" s="15" t="str">
-        <x:v>postback</x:v>
-      </x:c>
-      <x:c r="D1" s="15" t="str">
-        <x:v>attachment</x:v>
-      </x:c>
-      <x:c r="E1" s="15" t="str">
-        <x:v>server_authenticated</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="16" t="str">
-        <x:v>web</x:v>
-      </x:c>
-      <x:c r="B2" s="17" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C2" s="17" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D2" s="17" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E2" s="17" t="b">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="16" t="str">
-        <x:v>whatsapp</x:v>
-      </x:c>
-      <x:c r="B3" s="17" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C3" s="17" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D3" s="17" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E3" s="17" t="b">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="16" t="str">
-        <x:v>email</x:v>
-      </x:c>
-      <x:c r="B4" s="17" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C4" s="17" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D4" s="17" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E4" s="17" t="b">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="16" t="str">
-        <x:v>sms</x:v>
-      </x:c>
-      <x:c r="B5" s="17" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C5" s="17" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D5" s="17" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E5" s="17" t="b">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="16" t="str">
-        <x:v>voice</x:v>
-      </x:c>
-      <x:c r="B6" s="17" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C6" s="17" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D6" s="17" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E6" s="17" t="b">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R985ab9ceeb9f4913"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a43975eeff34163"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>